<commit_message>
Predict the quencher properties with the new model
quencher_properties_ml.xlsx is rerun with the full-data trial-55 model, and
exp_dataset_ent and the benchmark are rebuilt from it. Only the ML columns of
the dataset and the ML rows of the benchmark results change; the pairs and
everything computed from DFT are unchanged. The ML timing table is not rerun.
</commit_message>
<xml_diff>
--- a/data/computational_data_processed/quencher_properties_ml.xlsx
+++ b/data/computational_data_processed/quencher_properties_ml.xlsx
@@ -568,22 +568,22 @@
         </is>
       </c>
       <c r="F3" s="7" t="n">
-        <v>60.09</v>
+        <v>60.58</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>1.41</v>
+        <v>1.12</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>13.33</v>
+        <v>13.15</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>1.15</v>
+        <v>0.73</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>12.03</v>
+        <v>12.62</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>1.2</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="4">
@@ -606,22 +606,22 @@
         </is>
       </c>
       <c r="F4" s="7" t="n">
-        <v>53.28</v>
+        <v>52.08</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>2.3</v>
+        <v>1.5</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>81.06999999999999</v>
+        <v>94</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>22.7</v>
+        <v>9.06</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>23.17</v>
+        <v>24.39</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>4.56</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="5">
@@ -644,22 +644,22 @@
         </is>
       </c>
       <c r="F5" s="7" t="n">
-        <v>60.72</v>
+        <v>59.62</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>1.67</v>
+        <v>1.37</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>32.46</v>
+        <v>30.75</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>3.09</v>
+        <v>2.22</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>19.18</v>
+        <v>19.07</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>2.82</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="6">
@@ -682,22 +682,22 @@
         </is>
       </c>
       <c r="F6" s="7" t="n">
-        <v>67.56999999999999</v>
+        <v>67.95999999999999</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>1.25</v>
+        <v>0.98</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>15.43</v>
+        <v>16.32</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>2.12</v>
+        <v>2.4</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>11.52</v>
+        <v>11.37</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>1.34</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="7">
@@ -720,22 +720,22 @@
         </is>
       </c>
       <c r="F7" s="7" t="n">
-        <v>58.52</v>
+        <v>59.21</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>2.62</v>
+        <v>1.12</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>11.79</v>
+        <v>13.02</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>1.48</v>
+        <v>0.77</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>10.2</v>
+        <v>11.47</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>1.7</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="8">
@@ -758,22 +758,22 @@
         </is>
       </c>
       <c r="F8" s="7" t="n">
-        <v>60.48</v>
+        <v>60.62</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>1.38</v>
+        <v>1.03</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>13.44</v>
+        <v>13.07</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>1.08</v>
+        <v>0.68</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>11.4</v>
+        <v>11.38</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>1.64</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="9">
@@ -796,22 +796,22 @@
         </is>
       </c>
       <c r="F9" s="7" t="n">
-        <v>59.74</v>
+        <v>59.51</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>1.64</v>
+        <v>1.18</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>11.06</v>
+        <v>11.66</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>1.29</v>
+        <v>0.79</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>9.140000000000001</v>
+        <v>10.02</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>1.02</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="10">
@@ -834,22 +834,22 @@
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>47.02</v>
+        <v>49.07</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>2.83</v>
+        <v>2.37</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>58.47</v>
+        <v>59.18</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>5.03</v>
+        <v>4.64</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>31.47</v>
+        <v>33.77</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>5.58</v>
+        <v>4.33</v>
       </c>
     </row>
     <row r="11">
@@ -872,22 +872,22 @@
         </is>
       </c>
       <c r="F11" s="7" t="n">
-        <v>57.02</v>
+        <v>57.68</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>2.26</v>
+        <v>1.57</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>17.53</v>
+        <v>18.33</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>2.14</v>
+        <v>2.29</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>13.33</v>
+        <v>14.89</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>1.95</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="12">
@@ -910,22 +910,22 @@
         </is>
       </c>
       <c r="F12" s="7" t="n">
-        <v>72.2</v>
+        <v>72.84</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>2.92</v>
+        <v>1.54</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>28.64</v>
+        <v>24.37</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>8.720000000000001</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>13.73</v>
+        <v>16.3</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>3.81</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="13">
@@ -948,22 +948,22 @@
         </is>
       </c>
       <c r="F13" s="7" t="n">
-        <v>75.59999999999999</v>
+        <v>76.76000000000001</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>4.76</v>
+        <v>3.59</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>28.87</v>
+        <v>34.17</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>10.59</v>
+        <v>7.14</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>17.34</v>
+        <v>25.57</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>7.36</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
@@ -986,22 +986,22 @@
         </is>
       </c>
       <c r="F14" s="7" t="n">
-        <v>53.33</v>
+        <v>56.61</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>3.94</v>
+        <v>1.96</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>21.08</v>
+        <v>16.12</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>5.86</v>
+        <v>2.27</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>17.27</v>
+        <v>12.83</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>3.59</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="15">
@@ -1024,22 +1024,22 @@
         </is>
       </c>
       <c r="F15" s="7" t="n">
-        <v>57.05</v>
+        <v>56.89</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>3.5</v>
+        <v>1.62</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>19.05</v>
+        <v>19.52</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>2.98</v>
+        <v>1.52</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>14.48</v>
+        <v>14.91</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>1.65</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="16">
@@ -1062,22 +1062,22 @@
         </is>
       </c>
       <c r="F16" s="7" t="n">
-        <v>53.83</v>
+        <v>53.99</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>2.21</v>
+        <v>1.52</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>91.58</v>
+        <v>95.19</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>9.140000000000001</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>29.9</v>
+        <v>30.32</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>5.1</v>
+        <v>6.62</v>
       </c>
     </row>
     <row r="17">
@@ -1100,22 +1100,22 @@
         </is>
       </c>
       <c r="F17" s="7" t="n">
-        <v>61.23</v>
+        <v>62.65</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>3.06</v>
+        <v>1.89</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>17.14</v>
+        <v>17.42</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>2</v>
+        <v>1.23</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>14.11</v>
+        <v>14.5</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>1.53</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="18">
@@ -1138,22 +1138,22 @@
         </is>
       </c>
       <c r="F18" s="7" t="n">
-        <v>56.78</v>
+        <v>56.22</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>1.95</v>
+        <v>1.5</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>11.03</v>
+        <v>10.64</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>1.33</v>
+        <v>1.04</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>9.460000000000001</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="19">
@@ -1176,22 +1176,22 @@
         </is>
       </c>
       <c r="F19" s="7" t="n">
-        <v>79.86</v>
+        <v>80.51000000000001</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>1.92</v>
+        <v>1.15</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>19.64</v>
+        <v>15</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>9.789999999999999</v>
+        <v>2.43</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>12.62</v>
+        <v>13.84</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>4.02</v>
+        <v>7.78</v>
       </c>
     </row>
     <row r="20">
@@ -1214,22 +1214,22 @@
         </is>
       </c>
       <c r="F20" s="7" t="n">
-        <v>54.59</v>
+        <v>52.27</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>2.88</v>
+        <v>2.5</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>23.57</v>
+        <v>21.83</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>4.11</v>
+        <v>2.46</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>17.6</v>
+        <v>17.82</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>2</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="21">
@@ -1252,22 +1252,22 @@
         </is>
       </c>
       <c r="F21" s="7" t="n">
-        <v>46.52</v>
+        <v>49.85</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>3.14</v>
+        <v>2.31</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>55.07</v>
+        <v>59.37</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>5.18</v>
+        <v>4.72</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>41.93</v>
+        <v>33.75</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>9.19</v>
+        <v>4.64</v>
       </c>
     </row>
     <row r="22">
@@ -1290,22 +1290,22 @@
         </is>
       </c>
       <c r="F22" s="7" t="n">
-        <v>61.15</v>
+        <v>61.1</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>1.29</v>
+        <v>1</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>12.68</v>
+        <v>12.09</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>1.06</v>
+        <v>0.59</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>10.78</v>
+        <v>10.63</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>1.21</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="23">
@@ -1328,22 +1328,22 @@
         </is>
       </c>
       <c r="F23" s="7" t="n">
-        <v>68.34999999999999</v>
+        <v>68.33</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>1.37</v>
+        <v>0.99</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>13.21</v>
+        <v>13.35</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>1.41</v>
+        <v>0.79</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>9.66</v>
+        <v>10.17</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>0.89</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="24">
@@ -1366,22 +1366,22 @@
         </is>
       </c>
       <c r="F24" s="7" t="n">
-        <v>60.79</v>
+        <v>63.41</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>2.09</v>
+        <v>1.97</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>21.61</v>
+        <v>20.36</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>6.04</v>
+        <v>2.57</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>17.97</v>
+        <v>17.52</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>3.6</v>
+        <v>3.88</v>
       </c>
     </row>
     <row r="25">
@@ -1404,22 +1404,22 @@
         </is>
       </c>
       <c r="F25" s="7" t="n">
-        <v>61.32</v>
+        <v>60.93</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>1.31</v>
+        <v>1.05</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>13.55</v>
+        <v>12.48</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>1.05</v>
+        <v>0.84</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>10.45</v>
+        <v>10.1</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>0.78</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="26">
@@ -1442,22 +1442,22 @@
         </is>
       </c>
       <c r="F26" s="7" t="n">
-        <v>63.44</v>
+        <v>63.33</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>1.26</v>
+        <v>1.09</v>
       </c>
       <c r="H26" s="7" t="n">
-        <v>14.62</v>
+        <v>13.46</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>1.41</v>
+        <v>0.87</v>
       </c>
       <c r="J26" s="7" t="n">
-        <v>11.26</v>
+        <v>10.98</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>1.04</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="27">
@@ -1480,22 +1480,22 @@
         </is>
       </c>
       <c r="F27" s="7" t="n">
-        <v>60.18</v>
+        <v>61.53</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>1.76</v>
+        <v>1.18</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>37.69</v>
+        <v>38.85</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>3.46</v>
+        <v>2.67</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>16.62</v>
+        <v>17.26</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>1.8</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="28">
@@ -1518,22 +1518,22 @@
         </is>
       </c>
       <c r="F28" s="7" t="n">
-        <v>59.67</v>
+        <v>60.82</v>
       </c>
       <c r="G28" s="7" t="n">
-        <v>2.08</v>
+        <v>1.79</v>
       </c>
       <c r="H28" s="7" t="n">
-        <v>40.43</v>
+        <v>43.12</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>3.95</v>
+        <v>3.71</v>
       </c>
       <c r="J28" s="7" t="n">
-        <v>22.53</v>
+        <v>22.1</v>
       </c>
       <c r="K28" s="7" t="n">
-        <v>3.06</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="29">
@@ -1556,22 +1556,22 @@
         </is>
       </c>
       <c r="F29" s="7" t="n">
-        <v>61.13</v>
+        <v>59.21</v>
       </c>
       <c r="G29" s="7" t="n">
-        <v>1.47</v>
+        <v>1.19</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>37.66</v>
+        <v>36.69</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>2.46</v>
+        <v>2.12</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>15.92</v>
+        <v>15.55</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>1.53</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="30">
@@ -1594,22 +1594,22 @@
         </is>
       </c>
       <c r="F30" s="7" t="n">
-        <v>59.16</v>
+        <v>57.53</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>2.09</v>
+        <v>1.41</v>
       </c>
       <c r="H30" s="7" t="n">
-        <v>16.42</v>
+        <v>14.75</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>1.48</v>
+        <v>1.22</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>9.66</v>
+        <v>8.91</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>1.61</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="31">
@@ -1632,22 +1632,22 @@
         </is>
       </c>
       <c r="F31" s="7" t="n">
-        <v>58.95</v>
+        <v>59.85</v>
       </c>
       <c r="G31" s="7" t="n">
-        <v>3.71</v>
+        <v>2.47</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>32.62</v>
+        <v>26.44</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>13.87</v>
+        <v>5.76</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>19.05</v>
+        <v>19.83</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>2.78</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="32">
@@ -1670,22 +1670,22 @@
         </is>
       </c>
       <c r="F32" s="7" t="n">
-        <v>44.43</v>
+        <v>43.94</v>
       </c>
       <c r="G32" s="7" t="n">
-        <v>2.63</v>
+        <v>2.05</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>63.53</v>
+        <v>65.23</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>7.8</v>
+        <v>6.9</v>
       </c>
       <c r="J32" s="7" t="n">
-        <v>18.37</v>
+        <v>18.81</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>2.3</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="33">
@@ -1708,22 +1708,22 @@
         </is>
       </c>
       <c r="F33" s="7" t="n">
-        <v>76.87</v>
+        <v>77.93000000000001</v>
       </c>
       <c r="G33" s="7" t="n">
-        <v>1.22</v>
+        <v>1.01</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>12.8</v>
+        <v>15.51</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>2.92</v>
+        <v>7.2</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>10.19</v>
+        <v>10.9</v>
       </c>
       <c r="K33" s="7" t="n">
-        <v>2.54</v>
+        <v>3.57</v>
       </c>
     </row>
     <row r="34">
@@ -1746,22 +1746,22 @@
         </is>
       </c>
       <c r="F34" s="7" t="n">
-        <v>54.89</v>
+        <v>53.68</v>
       </c>
       <c r="G34" s="7" t="n">
-        <v>3.04</v>
+        <v>2.12</v>
       </c>
       <c r="H34" s="7" t="n">
-        <v>37.24</v>
+        <v>35.54</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>5.1</v>
+        <v>4.31</v>
       </c>
       <c r="J34" s="7" t="n">
-        <v>15.91</v>
+        <v>15.14</v>
       </c>
       <c r="K34" s="7" t="n">
-        <v>2.32</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="35">
@@ -1784,22 +1784,22 @@
         </is>
       </c>
       <c r="F35" s="7" t="n">
-        <v>60.94</v>
+        <v>59.1</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>2.83</v>
+        <v>2.54</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>31.31</v>
+        <v>29.5</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>5.75</v>
+        <v>7.86</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>13.14</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>3.74</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="36">
@@ -1822,22 +1822,22 @@
         </is>
       </c>
       <c r="F36" s="7" t="n">
-        <v>46.58</v>
+        <v>46.34</v>
       </c>
       <c r="G36" s="7" t="n">
-        <v>2.78</v>
+        <v>2.37</v>
       </c>
       <c r="H36" s="7" t="n">
-        <v>73.79000000000001</v>
+        <v>69.58</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>6.18</v>
+        <v>4.55</v>
       </c>
       <c r="J36" s="7" t="n">
-        <v>37.41</v>
+        <v>37.52</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>5.8</v>
+        <v>3.79</v>
       </c>
     </row>
     <row r="37">
@@ -1860,22 +1860,22 @@
         </is>
       </c>
       <c r="F37" s="7" t="n">
-        <v>39.61</v>
+        <v>38.94</v>
       </c>
       <c r="G37" s="7" t="n">
-        <v>2.86</v>
+        <v>2.34</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>57.41</v>
+        <v>58.81</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>5.69</v>
+        <v>4.06</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>30.13</v>
+        <v>31.72</v>
       </c>
       <c r="K37" s="7" t="n">
-        <v>4.78</v>
+        <v>3.16</v>
       </c>
     </row>
     <row r="38">
@@ -1898,22 +1898,22 @@
         </is>
       </c>
       <c r="F38" s="7" t="n">
-        <v>64.69</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="G38" s="7" t="n">
-        <v>1.76</v>
+        <v>1.2</v>
       </c>
       <c r="H38" s="7" t="n">
-        <v>12</v>
+        <v>11.42</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>1.28</v>
+        <v>0.84</v>
       </c>
       <c r="J38" s="7" t="n">
-        <v>8.08</v>
+        <v>7.24</v>
       </c>
       <c r="K38" s="7" t="n">
-        <v>1.39</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="39">
@@ -1936,22 +1936,22 @@
         </is>
       </c>
       <c r="F39" s="7" t="n">
-        <v>47.85</v>
+        <v>49.05</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>2.48</v>
+        <v>1.88</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>77.76000000000001</v>
+        <v>78.2</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>6.4</v>
+        <v>8.01</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>27.12</v>
+        <v>27.49</v>
       </c>
       <c r="K39" s="7" t="n">
-        <v>3.51</v>
+        <v>3.96</v>
       </c>
     </row>
     <row r="40">
@@ -1974,22 +1974,22 @@
         </is>
       </c>
       <c r="F40" s="7" t="n">
-        <v>55.65</v>
+        <v>56.32</v>
       </c>
       <c r="G40" s="7" t="n">
-        <v>3.84</v>
+        <v>3.01</v>
       </c>
       <c r="H40" s="7" t="n">
-        <v>27.1</v>
+        <v>22.1</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>21.35</v>
+        <v>6.79</v>
       </c>
       <c r="J40" s="7" t="n">
-        <v>17.49</v>
+        <v>15.33</v>
       </c>
       <c r="K40" s="7" t="n">
-        <v>6.79</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="41">
@@ -2012,22 +2012,22 @@
         </is>
       </c>
       <c r="F41" s="7" t="n">
-        <v>55.36</v>
+        <v>55.67</v>
       </c>
       <c r="G41" s="7" t="n">
-        <v>2.34</v>
+        <v>1.72</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>17.83</v>
+        <v>17.45</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>1.69</v>
+        <v>2.06</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>13.03</v>
+        <v>13.6</v>
       </c>
       <c r="K41" s="7" t="n">
-        <v>1.26</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="42">
@@ -2050,22 +2050,22 @@
         </is>
       </c>
       <c r="F42" s="7" t="n">
-        <v>63.52</v>
+        <v>64.03</v>
       </c>
       <c r="G42" s="7" t="n">
-        <v>1.69</v>
+        <v>1.21</v>
       </c>
       <c r="H42" s="7" t="n">
-        <v>17.35</v>
+        <v>17.51</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>1.19</v>
+        <v>0.82</v>
       </c>
       <c r="J42" s="7" t="n">
-        <v>14.02</v>
+        <v>14.78</v>
       </c>
       <c r="K42" s="7" t="n">
-        <v>1.31</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="43">
@@ -2088,22 +2088,22 @@
         </is>
       </c>
       <c r="F43" s="7" t="n">
-        <v>52.17</v>
+        <v>51.51</v>
       </c>
       <c r="G43" s="7" t="n">
-        <v>2.18</v>
+        <v>1.71</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>91.56999999999999</v>
+        <v>88.14</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>8.970000000000001</v>
+        <v>7.84</v>
       </c>
       <c r="J43" s="7" t="n">
-        <v>28.77</v>
+        <v>26.8</v>
       </c>
       <c r="K43" s="7" t="n">
-        <v>4.81</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="44">
@@ -2126,22 +2126,22 @@
         </is>
       </c>
       <c r="F44" s="7" t="n">
-        <v>59.15</v>
+        <v>59.38</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>1.85</v>
+        <v>1.56</v>
       </c>
       <c r="H44" s="7" t="n">
-        <v>12.54</v>
+        <v>11.59</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>1.35</v>
+        <v>1.28</v>
       </c>
       <c r="J44" s="7" t="n">
-        <v>8.08</v>
+        <v>7.08</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>2.26</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="45">
@@ -2164,22 +2164,22 @@
         </is>
       </c>
       <c r="F45" s="7" t="n">
-        <v>58.57</v>
+        <v>59.42</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>1.53</v>
+        <v>1.15</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>13.78</v>
+        <v>13.46</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>1.14</v>
+        <v>0.83</v>
       </c>
       <c r="J45" s="7" t="n">
-        <v>8.82</v>
+        <v>8.83</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>0.89</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="46">
@@ -2202,22 +2202,22 @@
         </is>
       </c>
       <c r="F46" s="7" t="n">
-        <v>65.62</v>
+        <v>65.59</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>1.95</v>
+        <v>1.29</v>
       </c>
       <c r="H46" s="7" t="n">
-        <v>11.21</v>
+        <v>10.34</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>2.24</v>
+        <v>2.59</v>
       </c>
       <c r="J46" s="7" t="n">
-        <v>14.45</v>
+        <v>16.15</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>4.06</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="47">
@@ -2240,22 +2240,22 @@
         </is>
       </c>
       <c r="F47" s="7" t="n">
-        <v>77.23</v>
+        <v>75.45999999999999</v>
       </c>
       <c r="G47" s="7" t="n">
-        <v>3.89</v>
+        <v>6.63</v>
       </c>
       <c r="H47" s="7" t="n">
-        <v>48.87</v>
+        <v>19.67</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>16.75</v>
+        <v>15.86</v>
       </c>
       <c r="J47" s="7" t="n">
-        <v>20.11</v>
+        <v>11.67</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>8.17</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="48">
@@ -2278,22 +2278,22 @@
         </is>
       </c>
       <c r="F48" s="7" t="n">
-        <v>58.33</v>
+        <v>63</v>
       </c>
       <c r="G48" s="7" t="n">
-        <v>4.09</v>
+        <v>3</v>
       </c>
       <c r="H48" s="7" t="n">
         <v>21.73</v>
       </c>
       <c r="I48" s="7" t="n">
-        <v>3.89</v>
+        <v>2.98</v>
       </c>
       <c r="J48" s="7" t="n">
-        <v>17.29</v>
+        <v>18.53</v>
       </c>
       <c r="K48" s="7" t="n">
-        <v>3.06</v>
+        <v>2.77</v>
       </c>
     </row>
     <row r="49">
@@ -2316,22 +2316,22 @@
         </is>
       </c>
       <c r="F49" s="7" t="n">
-        <v>60.61</v>
+        <v>61.53</v>
       </c>
       <c r="G49" s="7" t="n">
-        <v>1.37</v>
+        <v>1.13</v>
       </c>
       <c r="H49" s="7" t="n">
-        <v>12.6</v>
+        <v>12.22</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>1.02</v>
+        <v>0.8</v>
       </c>
       <c r="J49" s="7" t="n">
-        <v>10.23</v>
+        <v>10.16</v>
       </c>
       <c r="K49" s="7" t="n">
-        <v>0.96</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="50">
@@ -2354,22 +2354,22 @@
         </is>
       </c>
       <c r="F50" s="7" t="n">
-        <v>59.93</v>
+        <v>64.5</v>
       </c>
       <c r="G50" s="7" t="n">
-        <v>3.75</v>
+        <v>1.88</v>
       </c>
       <c r="H50" s="7" t="n">
-        <v>42.93</v>
+        <v>14.32</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>17.64</v>
+        <v>10.57</v>
       </c>
       <c r="J50" s="7" t="n">
-        <v>15.87</v>
+        <v>12.34</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>3.47</v>
+        <v>4.81</v>
       </c>
     </row>
   </sheetData>
@@ -2539,7 +2539,7 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>ml/data/model.pt: triplet_energy_adiabatic</t>
+          <t>ml/data/model_final.pt: triplet_energy_adiabatic</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2566,7 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>ml/data/model.pt: triplet_energy_adiabatic_uncertainty</t>
+          <t>ml/data/model_final.pt: triplet_energy_adiabatic_uncertainty</t>
         </is>
       </c>
     </row>
@@ -2593,7 +2593,7 @@
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>ml/data/model.pt: lamda_S_T</t>
+          <t>ml/data/model_final.pt: lamda_S_T</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>ml/data/model.pt: lamda_S_T_uncertainty</t>
+          <t>ml/data/model_final.pt: lamda_S_T_uncertainty</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2647,7 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>ml/data/model.pt: lamda_T_S</t>
+          <t>ml/data/model_final.pt: lamda_T_S</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>ml/data/model.pt: lamda_T_S_uncertainty</t>
+          <t>ml/data/model_final.pt: lamda_T_S_uncertainty</t>
         </is>
       </c>
     </row>
@@ -2699,7 +2699,7 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>network in ml/data/model.pt. The same three quantities from DFT are in</t>
+          <t>network in ml/data/model_final.pt. The same three quantities from DFT are in</t>
         </is>
       </c>
       <c r="B14" s="9" t="n"/>

</xml_diff>